<commit_message>
fix: resolve security report generator syntax error and add Android Appium E2E pipeline
</commit_message>
<xml_diff>
--- a/security_automation/Test Results/Excel/Execution_Report.xlsx
+++ b/security_automation/Test Results/Excel/Execution_Report.xlsx
@@ -77,7 +77,7 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>2026-08-06T05:42:03.690Z</t>
+    <t>2026-08-06T06:17:25.015Z</t>
   </si>
   <si>
     <t>TC_SEC_SQLI_002</t>
@@ -1001,9 +1001,6 @@
     <t>Verify Vulnerability Defense: CSRF &amp; Origin Security Check #2</t>
   </si>
   <si>
-    <t>2026-08-06T05:42:03.691Z</t>
-  </si>
-  <si>
     <t>TC_SEC_CSRF_003</t>
   </si>
   <si>
@@ -1223,6 +1220,9 @@
     <t>Verify Vulnerability Defense: API Security &amp; OWASP Top 10 Check #8</t>
   </si>
   <si>
+    <t>2026-08-06T06:17:25.016Z</t>
+  </si>
+  <si>
     <t>TC_SEC_API_009</t>
   </si>
   <si>
@@ -1925,7 +1925,7 @@
     <t>Execution Timestamp</t>
   </si>
   <si>
-    <t>Thu, 06 Aug 2026 05:42:03 GMT</t>
+    <t>Thu, 06 Aug 2026 06:17:24 GMT</t>
   </si>
   <si>
     <t>Security Scanner</t>
@@ -7713,15 +7713,15 @@
         <v>19</v>
       </c>
       <c r="K153" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="154" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
+        <v>328</v>
+      </c>
+      <c r="B154" t="s">
         <v>329</v>
-      </c>
-      <c r="B154" t="s">
-        <v>330</v>
       </c>
       <c r="C154" t="s">
         <v>325</v>
@@ -7748,15 +7748,15 @@
         <v>19</v>
       </c>
       <c r="K154" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="155" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
+        <v>330</v>
+      </c>
+      <c r="B155" t="s">
         <v>331</v>
-      </c>
-      <c r="B155" t="s">
-        <v>332</v>
       </c>
       <c r="C155" t="s">
         <v>325</v>
@@ -7783,15 +7783,15 @@
         <v>19</v>
       </c>
       <c r="K155" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="156" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
+        <v>332</v>
+      </c>
+      <c r="B156" t="s">
         <v>333</v>
-      </c>
-      <c r="B156" t="s">
-        <v>334</v>
       </c>
       <c r="C156" t="s">
         <v>325</v>
@@ -7818,15 +7818,15 @@
         <v>19</v>
       </c>
       <c r="K156" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="157" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
+        <v>334</v>
+      </c>
+      <c r="B157" t="s">
         <v>335</v>
-      </c>
-      <c r="B157" t="s">
-        <v>336</v>
       </c>
       <c r="C157" t="s">
         <v>325</v>
@@ -7853,15 +7853,15 @@
         <v>19</v>
       </c>
       <c r="K157" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="158" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
+        <v>336</v>
+      </c>
+      <c r="B158" t="s">
         <v>337</v>
-      </c>
-      <c r="B158" t="s">
-        <v>338</v>
       </c>
       <c r="C158" t="s">
         <v>325</v>
@@ -7888,15 +7888,15 @@
         <v>19</v>
       </c>
       <c r="K158" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="159" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
+        <v>338</v>
+      </c>
+      <c r="B159" t="s">
         <v>339</v>
-      </c>
-      <c r="B159" t="s">
-        <v>340</v>
       </c>
       <c r="C159" t="s">
         <v>325</v>
@@ -7923,15 +7923,15 @@
         <v>19</v>
       </c>
       <c r="K159" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="160" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
+        <v>340</v>
+      </c>
+      <c r="B160" t="s">
         <v>341</v>
-      </c>
-      <c r="B160" t="s">
-        <v>342</v>
       </c>
       <c r="C160" t="s">
         <v>325</v>
@@ -7958,15 +7958,15 @@
         <v>19</v>
       </c>
       <c r="K160" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="161" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
+        <v>342</v>
+      </c>
+      <c r="B161" t="s">
         <v>343</v>
-      </c>
-      <c r="B161" t="s">
-        <v>344</v>
       </c>
       <c r="C161" t="s">
         <v>325</v>
@@ -7993,15 +7993,15 @@
         <v>19</v>
       </c>
       <c r="K161" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="162" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
+        <v>344</v>
+      </c>
+      <c r="B162" t="s">
         <v>345</v>
-      </c>
-      <c r="B162" t="s">
-        <v>346</v>
       </c>
       <c r="C162" t="s">
         <v>325</v>
@@ -8028,15 +8028,15 @@
         <v>19</v>
       </c>
       <c r="K162" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="163" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
+        <v>346</v>
+      </c>
+      <c r="B163" t="s">
         <v>347</v>
-      </c>
-      <c r="B163" t="s">
-        <v>348</v>
       </c>
       <c r="C163" t="s">
         <v>325</v>
@@ -8063,15 +8063,15 @@
         <v>19</v>
       </c>
       <c r="K163" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="164" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
+        <v>348</v>
+      </c>
+      <c r="B164" t="s">
         <v>349</v>
-      </c>
-      <c r="B164" t="s">
-        <v>350</v>
       </c>
       <c r="C164" t="s">
         <v>325</v>
@@ -8098,15 +8098,15 @@
         <v>19</v>
       </c>
       <c r="K164" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="165" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
+        <v>350</v>
+      </c>
+      <c r="B165" t="s">
         <v>351</v>
-      </c>
-      <c r="B165" t="s">
-        <v>352</v>
       </c>
       <c r="C165" t="s">
         <v>325</v>
@@ -8133,15 +8133,15 @@
         <v>19</v>
       </c>
       <c r="K165" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="166" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
+        <v>352</v>
+      </c>
+      <c r="B166" t="s">
         <v>353</v>
-      </c>
-      <c r="B166" t="s">
-        <v>354</v>
       </c>
       <c r="C166" t="s">
         <v>325</v>
@@ -8168,15 +8168,15 @@
         <v>19</v>
       </c>
       <c r="K166" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="167" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
+        <v>354</v>
+      </c>
+      <c r="B167" t="s">
         <v>355</v>
-      </c>
-      <c r="B167" t="s">
-        <v>356</v>
       </c>
       <c r="C167" t="s">
         <v>325</v>
@@ -8203,15 +8203,15 @@
         <v>19</v>
       </c>
       <c r="K167" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="168" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
+        <v>356</v>
+      </c>
+      <c r="B168" t="s">
         <v>357</v>
-      </c>
-      <c r="B168" t="s">
-        <v>358</v>
       </c>
       <c r="C168" t="s">
         <v>325</v>
@@ -8238,15 +8238,15 @@
         <v>19</v>
       </c>
       <c r="K168" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="169" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
+        <v>358</v>
+      </c>
+      <c r="B169" t="s">
         <v>359</v>
-      </c>
-      <c r="B169" t="s">
-        <v>360</v>
       </c>
       <c r="C169" t="s">
         <v>325</v>
@@ -8273,15 +8273,15 @@
         <v>19</v>
       </c>
       <c r="K169" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="170" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
+        <v>360</v>
+      </c>
+      <c r="B170" t="s">
         <v>361</v>
-      </c>
-      <c r="B170" t="s">
-        <v>362</v>
       </c>
       <c r="C170" t="s">
         <v>325</v>
@@ -8308,15 +8308,15 @@
         <v>19</v>
       </c>
       <c r="K170" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="171" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
+        <v>362</v>
+      </c>
+      <c r="B171" t="s">
         <v>363</v>
-      </c>
-      <c r="B171" t="s">
-        <v>364</v>
       </c>
       <c r="C171" t="s">
         <v>325</v>
@@ -8343,15 +8343,15 @@
         <v>19</v>
       </c>
       <c r="K171" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="172" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
+        <v>364</v>
+      </c>
+      <c r="B172" t="s">
         <v>365</v>
-      </c>
-      <c r="B172" t="s">
-        <v>366</v>
       </c>
       <c r="C172" t="s">
         <v>325</v>
@@ -8378,15 +8378,15 @@
         <v>19</v>
       </c>
       <c r="K172" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="173" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
+        <v>366</v>
+      </c>
+      <c r="B173" t="s">
         <v>367</v>
-      </c>
-      <c r="B173" t="s">
-        <v>368</v>
       </c>
       <c r="C173" t="s">
         <v>325</v>
@@ -8413,15 +8413,15 @@
         <v>19</v>
       </c>
       <c r="K173" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="174" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
+        <v>368</v>
+      </c>
+      <c r="B174" t="s">
         <v>369</v>
-      </c>
-      <c r="B174" t="s">
-        <v>370</v>
       </c>
       <c r="C174" t="s">
         <v>325</v>
@@ -8448,15 +8448,15 @@
         <v>19</v>
       </c>
       <c r="K174" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="175" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
+        <v>370</v>
+      </c>
+      <c r="B175" t="s">
         <v>371</v>
-      </c>
-      <c r="B175" t="s">
-        <v>372</v>
       </c>
       <c r="C175" t="s">
         <v>325</v>
@@ -8483,15 +8483,15 @@
         <v>19</v>
       </c>
       <c r="K175" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="176" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
+        <v>372</v>
+      </c>
+      <c r="B176" t="s">
         <v>373</v>
-      </c>
-      <c r="B176" t="s">
-        <v>374</v>
       </c>
       <c r="C176" t="s">
         <v>325</v>
@@ -8518,15 +8518,15 @@
         <v>19</v>
       </c>
       <c r="K176" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="177" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
+        <v>374</v>
+      </c>
+      <c r="B177" t="s">
         <v>375</v>
-      </c>
-      <c r="B177" t="s">
-        <v>376</v>
       </c>
       <c r="C177" t="s">
         <v>325</v>
@@ -8553,15 +8553,15 @@
         <v>19</v>
       </c>
       <c r="K177" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="178" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
+        <v>376</v>
+      </c>
+      <c r="B178" t="s">
         <v>377</v>
-      </c>
-      <c r="B178" t="s">
-        <v>378</v>
       </c>
       <c r="C178" t="s">
         <v>325</v>
@@ -8588,15 +8588,15 @@
         <v>19</v>
       </c>
       <c r="K178" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="179" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
+        <v>378</v>
+      </c>
+      <c r="B179" t="s">
         <v>379</v>
-      </c>
-      <c r="B179" t="s">
-        <v>380</v>
       </c>
       <c r="C179" t="s">
         <v>325</v>
@@ -8623,15 +8623,15 @@
         <v>19</v>
       </c>
       <c r="K179" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="180" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
+        <v>380</v>
+      </c>
+      <c r="B180" t="s">
         <v>381</v>
-      </c>
-      <c r="B180" t="s">
-        <v>382</v>
       </c>
       <c r="C180" t="s">
         <v>325</v>
@@ -8658,15 +8658,15 @@
         <v>19</v>
       </c>
       <c r="K180" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="181" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
+        <v>382</v>
+      </c>
+      <c r="B181" t="s">
         <v>383</v>
-      </c>
-      <c r="B181" t="s">
-        <v>384</v>
       </c>
       <c r="C181" t="s">
         <v>325</v>
@@ -8693,19 +8693,19 @@
         <v>19</v>
       </c>
       <c r="K181" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="182" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
+        <v>384</v>
+      </c>
+      <c r="B182" t="s">
         <v>385</v>
       </c>
-      <c r="B182" t="s">
+      <c r="C182" t="s">
         <v>386</v>
       </c>
-      <c r="C182" t="s">
-        <v>387</v>
-      </c>
       <c r="D182" t="s">
         <v>14</v>
       </c>
@@ -8728,18 +8728,18 @@
         <v>19</v>
       </c>
       <c r="K182" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="183" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
+        <v>387</v>
+      </c>
+      <c r="B183" t="s">
         <v>388</v>
       </c>
-      <c r="B183" t="s">
-        <v>389</v>
-      </c>
       <c r="C183" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D183" t="s">
         <v>14</v>
@@ -8763,18 +8763,18 @@
         <v>19</v>
       </c>
       <c r="K183" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="184" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
+        <v>389</v>
+      </c>
+      <c r="B184" t="s">
         <v>390</v>
       </c>
-      <c r="B184" t="s">
-        <v>391</v>
-      </c>
       <c r="C184" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D184" t="s">
         <v>14</v>
@@ -8798,18 +8798,18 @@
         <v>19</v>
       </c>
       <c r="K184" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="185" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
+        <v>391</v>
+      </c>
+      <c r="B185" t="s">
         <v>392</v>
       </c>
-      <c r="B185" t="s">
-        <v>393</v>
-      </c>
       <c r="C185" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D185" t="s">
         <v>14</v>
@@ -8833,18 +8833,18 @@
         <v>19</v>
       </c>
       <c r="K185" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="186" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
+        <v>393</v>
+      </c>
+      <c r="B186" t="s">
         <v>394</v>
       </c>
-      <c r="B186" t="s">
-        <v>395</v>
-      </c>
       <c r="C186" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D186" t="s">
         <v>14</v>
@@ -8868,18 +8868,18 @@
         <v>19</v>
       </c>
       <c r="K186" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="187" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
+        <v>395</v>
+      </c>
+      <c r="B187" t="s">
         <v>396</v>
       </c>
-      <c r="B187" t="s">
-        <v>397</v>
-      </c>
       <c r="C187" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D187" t="s">
         <v>14</v>
@@ -8903,18 +8903,18 @@
         <v>19</v>
       </c>
       <c r="K187" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="188" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
+        <v>397</v>
+      </c>
+      <c r="B188" t="s">
         <v>398</v>
       </c>
-      <c r="B188" t="s">
-        <v>399</v>
-      </c>
       <c r="C188" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D188" t="s">
         <v>14</v>
@@ -8938,42 +8938,42 @@
         <v>19</v>
       </c>
       <c r="K188" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="189" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
+        <v>399</v>
+      </c>
+      <c r="B189" t="s">
         <v>400</v>
       </c>
-      <c r="B189" t="s">
+      <c r="C189" t="s">
+        <v>386</v>
+      </c>
+      <c r="D189" t="s">
+        <v>14</v>
+      </c>
+      <c r="E189" t="s">
+        <v>15</v>
+      </c>
+      <c r="F189" t="s">
+        <v>16</v>
+      </c>
+      <c r="G189" t="s">
+        <v>17</v>
+      </c>
+      <c r="H189" t="s">
+        <v>18</v>
+      </c>
+      <c r="I189" t="s">
+        <v>19</v>
+      </c>
+      <c r="J189" t="s">
+        <v>19</v>
+      </c>
+      <c r="K189" t="s">
         <v>401</v>
-      </c>
-      <c r="C189" t="s">
-        <v>387</v>
-      </c>
-      <c r="D189" t="s">
-        <v>14</v>
-      </c>
-      <c r="E189" t="s">
-        <v>15</v>
-      </c>
-      <c r="F189" t="s">
-        <v>16</v>
-      </c>
-      <c r="G189" t="s">
-        <v>17</v>
-      </c>
-      <c r="H189" t="s">
-        <v>18</v>
-      </c>
-      <c r="I189" t="s">
-        <v>19</v>
-      </c>
-      <c r="J189" t="s">
-        <v>19</v>
-      </c>
-      <c r="K189" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="190" spans="1:11" x14ac:dyDescent="0.25">
@@ -8984,7 +8984,7 @@
         <v>403</v>
       </c>
       <c r="C190" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D190" t="s">
         <v>14</v>
@@ -9008,7 +9008,7 @@
         <v>19</v>
       </c>
       <c r="K190" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="191" spans="1:11" x14ac:dyDescent="0.25">
@@ -9019,7 +9019,7 @@
         <v>405</v>
       </c>
       <c r="C191" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D191" t="s">
         <v>14</v>
@@ -9043,7 +9043,7 @@
         <v>19</v>
       </c>
       <c r="K191" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="192" spans="1:11" x14ac:dyDescent="0.25">
@@ -9054,7 +9054,7 @@
         <v>407</v>
       </c>
       <c r="C192" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D192" t="s">
         <v>14</v>
@@ -9078,7 +9078,7 @@
         <v>19</v>
       </c>
       <c r="K192" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="193" spans="1:11" x14ac:dyDescent="0.25">
@@ -9089,7 +9089,7 @@
         <v>409</v>
       </c>
       <c r="C193" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D193" t="s">
         <v>14</v>
@@ -9113,7 +9113,7 @@
         <v>19</v>
       </c>
       <c r="K193" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="194" spans="1:11" x14ac:dyDescent="0.25">
@@ -9124,7 +9124,7 @@
         <v>411</v>
       </c>
       <c r="C194" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D194" t="s">
         <v>14</v>
@@ -9148,7 +9148,7 @@
         <v>19</v>
       </c>
       <c r="K194" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="195" spans="1:11" x14ac:dyDescent="0.25">
@@ -9159,7 +9159,7 @@
         <v>413</v>
       </c>
       <c r="C195" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D195" t="s">
         <v>14</v>
@@ -9183,7 +9183,7 @@
         <v>19</v>
       </c>
       <c r="K195" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="196" spans="1:11" x14ac:dyDescent="0.25">
@@ -9194,7 +9194,7 @@
         <v>415</v>
       </c>
       <c r="C196" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D196" t="s">
         <v>14</v>
@@ -9218,7 +9218,7 @@
         <v>19</v>
       </c>
       <c r="K196" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="197" spans="1:11" x14ac:dyDescent="0.25">
@@ -9229,7 +9229,7 @@
         <v>417</v>
       </c>
       <c r="C197" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D197" t="s">
         <v>14</v>
@@ -9253,7 +9253,7 @@
         <v>19</v>
       </c>
       <c r="K197" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="198" spans="1:11" x14ac:dyDescent="0.25">
@@ -9264,7 +9264,7 @@
         <v>419</v>
       </c>
       <c r="C198" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D198" t="s">
         <v>14</v>
@@ -9288,7 +9288,7 @@
         <v>19</v>
       </c>
       <c r="K198" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="199" spans="1:11" x14ac:dyDescent="0.25">
@@ -9299,7 +9299,7 @@
         <v>421</v>
       </c>
       <c r="C199" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D199" t="s">
         <v>14</v>
@@ -9323,7 +9323,7 @@
         <v>19</v>
       </c>
       <c r="K199" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="200" spans="1:11" x14ac:dyDescent="0.25">
@@ -9334,7 +9334,7 @@
         <v>423</v>
       </c>
       <c r="C200" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D200" t="s">
         <v>14</v>
@@ -9358,7 +9358,7 @@
         <v>19</v>
       </c>
       <c r="K200" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="201" spans="1:11" x14ac:dyDescent="0.25">
@@ -9369,7 +9369,7 @@
         <v>425</v>
       </c>
       <c r="C201" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D201" t="s">
         <v>14</v>
@@ -9393,7 +9393,7 @@
         <v>19</v>
       </c>
       <c r="K201" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="202" spans="1:11" x14ac:dyDescent="0.25">
@@ -9404,7 +9404,7 @@
         <v>427</v>
       </c>
       <c r="C202" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D202" t="s">
         <v>14</v>
@@ -9428,7 +9428,7 @@
         <v>19</v>
       </c>
       <c r="K202" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="203" spans="1:11" x14ac:dyDescent="0.25">
@@ -9439,7 +9439,7 @@
         <v>429</v>
       </c>
       <c r="C203" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D203" t="s">
         <v>14</v>
@@ -9463,7 +9463,7 @@
         <v>19</v>
       </c>
       <c r="K203" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="204" spans="1:11" x14ac:dyDescent="0.25">
@@ -9474,7 +9474,7 @@
         <v>431</v>
       </c>
       <c r="C204" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D204" t="s">
         <v>14</v>
@@ -9498,7 +9498,7 @@
         <v>19</v>
       </c>
       <c r="K204" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="205" spans="1:11" x14ac:dyDescent="0.25">
@@ -9509,7 +9509,7 @@
         <v>433</v>
       </c>
       <c r="C205" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D205" t="s">
         <v>14</v>
@@ -9533,7 +9533,7 @@
         <v>19</v>
       </c>
       <c r="K205" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="206" spans="1:11" x14ac:dyDescent="0.25">
@@ -9544,7 +9544,7 @@
         <v>435</v>
       </c>
       <c r="C206" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D206" t="s">
         <v>14</v>
@@ -9568,7 +9568,7 @@
         <v>19</v>
       </c>
       <c r="K206" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="207" spans="1:11" x14ac:dyDescent="0.25">
@@ -9579,7 +9579,7 @@
         <v>437</v>
       </c>
       <c r="C207" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D207" t="s">
         <v>14</v>
@@ -9603,7 +9603,7 @@
         <v>19</v>
       </c>
       <c r="K207" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="208" spans="1:11" x14ac:dyDescent="0.25">
@@ -9614,7 +9614,7 @@
         <v>439</v>
       </c>
       <c r="C208" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D208" t="s">
         <v>14</v>
@@ -9638,7 +9638,7 @@
         <v>19</v>
       </c>
       <c r="K208" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="209" spans="1:11" x14ac:dyDescent="0.25">
@@ -9649,7 +9649,7 @@
         <v>441</v>
       </c>
       <c r="C209" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D209" t="s">
         <v>14</v>
@@ -9673,7 +9673,7 @@
         <v>19</v>
       </c>
       <c r="K209" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="210" spans="1:11" x14ac:dyDescent="0.25">
@@ -9684,7 +9684,7 @@
         <v>443</v>
       </c>
       <c r="C210" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D210" t="s">
         <v>14</v>
@@ -9708,7 +9708,7 @@
         <v>19</v>
       </c>
       <c r="K210" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="211" spans="1:11" x14ac:dyDescent="0.25">
@@ -9719,7 +9719,7 @@
         <v>445</v>
       </c>
       <c r="C211" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D211" t="s">
         <v>14</v>
@@ -9743,7 +9743,7 @@
         <v>19</v>
       </c>
       <c r="K211" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="212" spans="1:11" x14ac:dyDescent="0.25">
@@ -9778,7 +9778,7 @@
         <v>19</v>
       </c>
       <c r="K212" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="213" spans="1:11" x14ac:dyDescent="0.25">
@@ -9813,7 +9813,7 @@
         <v>19</v>
       </c>
       <c r="K213" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="214" spans="1:11" x14ac:dyDescent="0.25">
@@ -9848,7 +9848,7 @@
         <v>19</v>
       </c>
       <c r="K214" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="215" spans="1:11" x14ac:dyDescent="0.25">
@@ -9883,7 +9883,7 @@
         <v>19</v>
       </c>
       <c r="K215" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="216" spans="1:11" x14ac:dyDescent="0.25">
@@ -9918,7 +9918,7 @@
         <v>19</v>
       </c>
       <c r="K216" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="217" spans="1:11" x14ac:dyDescent="0.25">
@@ -9953,7 +9953,7 @@
         <v>19</v>
       </c>
       <c r="K217" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="218" spans="1:11" x14ac:dyDescent="0.25">
@@ -9988,7 +9988,7 @@
         <v>19</v>
       </c>
       <c r="K218" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="219" spans="1:11" x14ac:dyDescent="0.25">
@@ -10023,7 +10023,7 @@
         <v>19</v>
       </c>
       <c r="K219" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="220" spans="1:11" x14ac:dyDescent="0.25">
@@ -10058,7 +10058,7 @@
         <v>19</v>
       </c>
       <c r="K220" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="221" spans="1:11" x14ac:dyDescent="0.25">
@@ -10093,7 +10093,7 @@
         <v>19</v>
       </c>
       <c r="K221" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="222" spans="1:11" x14ac:dyDescent="0.25">
@@ -10128,7 +10128,7 @@
         <v>19</v>
       </c>
       <c r="K222" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="223" spans="1:11" x14ac:dyDescent="0.25">
@@ -10163,7 +10163,7 @@
         <v>19</v>
       </c>
       <c r="K223" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="224" spans="1:11" x14ac:dyDescent="0.25">
@@ -10198,7 +10198,7 @@
         <v>19</v>
       </c>
       <c r="K224" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="225" spans="1:11" x14ac:dyDescent="0.25">
@@ -10233,7 +10233,7 @@
         <v>19</v>
       </c>
       <c r="K225" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="226" spans="1:11" x14ac:dyDescent="0.25">
@@ -10268,7 +10268,7 @@
         <v>19</v>
       </c>
       <c r="K226" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="227" spans="1:11" x14ac:dyDescent="0.25">
@@ -10303,7 +10303,7 @@
         <v>19</v>
       </c>
       <c r="K227" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="228" spans="1:11" x14ac:dyDescent="0.25">
@@ -10338,7 +10338,7 @@
         <v>19</v>
       </c>
       <c r="K228" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="229" spans="1:11" x14ac:dyDescent="0.25">
@@ -10373,7 +10373,7 @@
         <v>19</v>
       </c>
       <c r="K229" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="230" spans="1:11" x14ac:dyDescent="0.25">
@@ -10408,7 +10408,7 @@
         <v>19</v>
       </c>
       <c r="K230" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="231" spans="1:11" x14ac:dyDescent="0.25">
@@ -10443,7 +10443,7 @@
         <v>19</v>
       </c>
       <c r="K231" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="232" spans="1:11" x14ac:dyDescent="0.25">
@@ -10478,7 +10478,7 @@
         <v>19</v>
       </c>
       <c r="K232" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="233" spans="1:11" x14ac:dyDescent="0.25">
@@ -10513,7 +10513,7 @@
         <v>19</v>
       </c>
       <c r="K233" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="234" spans="1:11" x14ac:dyDescent="0.25">
@@ -10548,7 +10548,7 @@
         <v>19</v>
       </c>
       <c r="K234" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="235" spans="1:11" x14ac:dyDescent="0.25">
@@ -10583,7 +10583,7 @@
         <v>19</v>
       </c>
       <c r="K235" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="236" spans="1:11" x14ac:dyDescent="0.25">
@@ -10618,7 +10618,7 @@
         <v>19</v>
       </c>
       <c r="K236" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="237" spans="1:11" x14ac:dyDescent="0.25">
@@ -10653,7 +10653,7 @@
         <v>19</v>
       </c>
       <c r="K237" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="238" spans="1:11" x14ac:dyDescent="0.25">
@@ -10688,7 +10688,7 @@
         <v>19</v>
       </c>
       <c r="K238" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="239" spans="1:11" x14ac:dyDescent="0.25">
@@ -10723,7 +10723,7 @@
         <v>19</v>
       </c>
       <c r="K239" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="240" spans="1:11" x14ac:dyDescent="0.25">
@@ -10758,7 +10758,7 @@
         <v>19</v>
       </c>
       <c r="K240" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="241" spans="1:11" x14ac:dyDescent="0.25">
@@ -10793,7 +10793,7 @@
         <v>19</v>
       </c>
       <c r="K241" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="242" spans="1:11" x14ac:dyDescent="0.25">
@@ -10828,7 +10828,7 @@
         <v>19</v>
       </c>
       <c r="K242" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="243" spans="1:11" x14ac:dyDescent="0.25">
@@ -10863,7 +10863,7 @@
         <v>19</v>
       </c>
       <c r="K243" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="244" spans="1:11" x14ac:dyDescent="0.25">
@@ -10898,7 +10898,7 @@
         <v>19</v>
       </c>
       <c r="K244" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="245" spans="1:11" x14ac:dyDescent="0.25">
@@ -10933,7 +10933,7 @@
         <v>19</v>
       </c>
       <c r="K245" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="246" spans="1:11" x14ac:dyDescent="0.25">
@@ -10968,7 +10968,7 @@
         <v>19</v>
       </c>
       <c r="K246" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="247" spans="1:11" x14ac:dyDescent="0.25">
@@ -11003,7 +11003,7 @@
         <v>19</v>
       </c>
       <c r="K247" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="248" spans="1:11" x14ac:dyDescent="0.25">
@@ -11038,7 +11038,7 @@
         <v>19</v>
       </c>
       <c r="K248" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="249" spans="1:11" x14ac:dyDescent="0.25">
@@ -11073,7 +11073,7 @@
         <v>19</v>
       </c>
       <c r="K249" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="250" spans="1:11" x14ac:dyDescent="0.25">
@@ -11108,7 +11108,7 @@
         <v>19</v>
       </c>
       <c r="K250" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="251" spans="1:11" x14ac:dyDescent="0.25">
@@ -11143,7 +11143,7 @@
         <v>19</v>
       </c>
       <c r="K251" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="252" spans="1:11" x14ac:dyDescent="0.25">
@@ -11178,7 +11178,7 @@
         <v>19</v>
       </c>
       <c r="K252" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="253" spans="1:11" x14ac:dyDescent="0.25">
@@ -11213,7 +11213,7 @@
         <v>19</v>
       </c>
       <c r="K253" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="254" spans="1:11" x14ac:dyDescent="0.25">
@@ -11248,7 +11248,7 @@
         <v>19</v>
       </c>
       <c r="K254" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="255" spans="1:11" x14ac:dyDescent="0.25">
@@ -11283,7 +11283,7 @@
         <v>19</v>
       </c>
       <c r="K255" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="256" spans="1:11" x14ac:dyDescent="0.25">
@@ -11318,7 +11318,7 @@
         <v>19</v>
       </c>
       <c r="K256" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="257" spans="1:11" x14ac:dyDescent="0.25">
@@ -11353,7 +11353,7 @@
         <v>19</v>
       </c>
       <c r="K257" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="258" spans="1:11" x14ac:dyDescent="0.25">
@@ -11388,7 +11388,7 @@
         <v>19</v>
       </c>
       <c r="K258" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="259" spans="1:11" x14ac:dyDescent="0.25">
@@ -11423,7 +11423,7 @@
         <v>19</v>
       </c>
       <c r="K259" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="260" spans="1:11" x14ac:dyDescent="0.25">
@@ -11458,7 +11458,7 @@
         <v>19</v>
       </c>
       <c r="K260" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="261" spans="1:11" x14ac:dyDescent="0.25">
@@ -11493,7 +11493,7 @@
         <v>19</v>
       </c>
       <c r="K261" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="262" spans="1:11" x14ac:dyDescent="0.25">
@@ -11528,7 +11528,7 @@
         <v>19</v>
       </c>
       <c r="K262" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="263" spans="1:11" x14ac:dyDescent="0.25">
@@ -11563,7 +11563,7 @@
         <v>19</v>
       </c>
       <c r="K263" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="264" spans="1:11" x14ac:dyDescent="0.25">
@@ -11598,7 +11598,7 @@
         <v>19</v>
       </c>
       <c r="K264" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="265" spans="1:11" x14ac:dyDescent="0.25">
@@ -11633,7 +11633,7 @@
         <v>19</v>
       </c>
       <c r="K265" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="266" spans="1:11" x14ac:dyDescent="0.25">
@@ -11668,7 +11668,7 @@
         <v>19</v>
       </c>
       <c r="K266" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="267" spans="1:11" x14ac:dyDescent="0.25">
@@ -11703,7 +11703,7 @@
         <v>19</v>
       </c>
       <c r="K267" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="268" spans="1:11" x14ac:dyDescent="0.25">
@@ -11738,7 +11738,7 @@
         <v>19</v>
       </c>
       <c r="K268" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="269" spans="1:11" x14ac:dyDescent="0.25">
@@ -11773,7 +11773,7 @@
         <v>19</v>
       </c>
       <c r="K269" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="270" spans="1:11" x14ac:dyDescent="0.25">
@@ -11808,7 +11808,7 @@
         <v>19</v>
       </c>
       <c r="K270" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="271" spans="1:11" x14ac:dyDescent="0.25">
@@ -11843,7 +11843,7 @@
         <v>19</v>
       </c>
       <c r="K271" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="272" spans="1:11" x14ac:dyDescent="0.25">
@@ -11878,7 +11878,7 @@
         <v>19</v>
       </c>
       <c r="K272" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="273" spans="1:11" x14ac:dyDescent="0.25">
@@ -11913,7 +11913,7 @@
         <v>19</v>
       </c>
       <c r="K273" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="274" spans="1:11" x14ac:dyDescent="0.25">
@@ -11948,7 +11948,7 @@
         <v>19</v>
       </c>
       <c r="K274" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="275" spans="1:11" x14ac:dyDescent="0.25">
@@ -11983,7 +11983,7 @@
         <v>19</v>
       </c>
       <c r="K275" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="276" spans="1:11" x14ac:dyDescent="0.25">
@@ -12018,7 +12018,7 @@
         <v>19</v>
       </c>
       <c r="K276" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="277" spans="1:11" x14ac:dyDescent="0.25">
@@ -12053,7 +12053,7 @@
         <v>19</v>
       </c>
       <c r="K277" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="278" spans="1:11" x14ac:dyDescent="0.25">
@@ -12088,7 +12088,7 @@
         <v>19</v>
       </c>
       <c r="K278" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="279" spans="1:11" x14ac:dyDescent="0.25">
@@ -12123,7 +12123,7 @@
         <v>19</v>
       </c>
       <c r="K279" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="280" spans="1:11" x14ac:dyDescent="0.25">
@@ -12158,7 +12158,7 @@
         <v>19</v>
       </c>
       <c r="K280" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="281" spans="1:11" x14ac:dyDescent="0.25">
@@ -12193,7 +12193,7 @@
         <v>19</v>
       </c>
       <c r="K281" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="282" spans="1:11" x14ac:dyDescent="0.25">
@@ -12228,7 +12228,7 @@
         <v>19</v>
       </c>
       <c r="K282" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="283" spans="1:11" x14ac:dyDescent="0.25">
@@ -12263,7 +12263,7 @@
         <v>19</v>
       </c>
       <c r="K283" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="284" spans="1:11" x14ac:dyDescent="0.25">
@@ -12298,7 +12298,7 @@
         <v>19</v>
       </c>
       <c r="K284" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="285" spans="1:11" x14ac:dyDescent="0.25">
@@ -12333,7 +12333,7 @@
         <v>19</v>
       </c>
       <c r="K285" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="286" spans="1:11" x14ac:dyDescent="0.25">
@@ -12368,7 +12368,7 @@
         <v>19</v>
       </c>
       <c r="K286" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="287" spans="1:11" x14ac:dyDescent="0.25">
@@ -12403,7 +12403,7 @@
         <v>19</v>
       </c>
       <c r="K287" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="288" spans="1:11" x14ac:dyDescent="0.25">
@@ -12438,7 +12438,7 @@
         <v>19</v>
       </c>
       <c r="K288" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="289" spans="1:11" x14ac:dyDescent="0.25">
@@ -12473,7 +12473,7 @@
         <v>19</v>
       </c>
       <c r="K289" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="290" spans="1:11" x14ac:dyDescent="0.25">
@@ -12508,7 +12508,7 @@
         <v>19</v>
       </c>
       <c r="K290" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="291" spans="1:11" x14ac:dyDescent="0.25">
@@ -12543,7 +12543,7 @@
         <v>19</v>
       </c>
       <c r="K291" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="292" spans="1:11" x14ac:dyDescent="0.25">
@@ -12578,7 +12578,7 @@
         <v>19</v>
       </c>
       <c r="K292" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="293" spans="1:11" x14ac:dyDescent="0.25">
@@ -12613,7 +12613,7 @@
         <v>19</v>
       </c>
       <c r="K293" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="294" spans="1:11" x14ac:dyDescent="0.25">
@@ -12648,7 +12648,7 @@
         <v>19</v>
       </c>
       <c r="K294" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="295" spans="1:11" x14ac:dyDescent="0.25">
@@ -12683,7 +12683,7 @@
         <v>19</v>
       </c>
       <c r="K295" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="296" spans="1:11" x14ac:dyDescent="0.25">
@@ -12718,7 +12718,7 @@
         <v>19</v>
       </c>
       <c r="K296" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="297" spans="1:11" x14ac:dyDescent="0.25">
@@ -12753,7 +12753,7 @@
         <v>19</v>
       </c>
       <c r="K297" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="298" spans="1:11" x14ac:dyDescent="0.25">
@@ -12788,7 +12788,7 @@
         <v>19</v>
       </c>
       <c r="K298" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="299" spans="1:11" x14ac:dyDescent="0.25">
@@ -12823,7 +12823,7 @@
         <v>19</v>
       </c>
       <c r="K299" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="300" spans="1:11" x14ac:dyDescent="0.25">
@@ -12858,7 +12858,7 @@
         <v>19</v>
       </c>
       <c r="K300" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="301" spans="1:11" x14ac:dyDescent="0.25">
@@ -12893,7 +12893,7 @@
         <v>19</v>
       </c>
       <c r="K301" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
   </sheetData>
@@ -18271,15 +18271,15 @@
         <v>19</v>
       </c>
       <c r="K153" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="154" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
+        <v>328</v>
+      </c>
+      <c r="B154" t="s">
         <v>329</v>
-      </c>
-      <c r="B154" t="s">
-        <v>330</v>
       </c>
       <c r="C154" t="s">
         <v>325</v>
@@ -18306,15 +18306,15 @@
         <v>19</v>
       </c>
       <c r="K154" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="155" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
+        <v>330</v>
+      </c>
+      <c r="B155" t="s">
         <v>331</v>
-      </c>
-      <c r="B155" t="s">
-        <v>332</v>
       </c>
       <c r="C155" t="s">
         <v>325</v>
@@ -18341,15 +18341,15 @@
         <v>19</v>
       </c>
       <c r="K155" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="156" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
+        <v>332</v>
+      </c>
+      <c r="B156" t="s">
         <v>333</v>
-      </c>
-      <c r="B156" t="s">
-        <v>334</v>
       </c>
       <c r="C156" t="s">
         <v>325</v>
@@ -18376,15 +18376,15 @@
         <v>19</v>
       </c>
       <c r="K156" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="157" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
+        <v>334</v>
+      </c>
+      <c r="B157" t="s">
         <v>335</v>
-      </c>
-      <c r="B157" t="s">
-        <v>336</v>
       </c>
       <c r="C157" t="s">
         <v>325</v>
@@ -18411,15 +18411,15 @@
         <v>19</v>
       </c>
       <c r="K157" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="158" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
+        <v>336</v>
+      </c>
+      <c r="B158" t="s">
         <v>337</v>
-      </c>
-      <c r="B158" t="s">
-        <v>338</v>
       </c>
       <c r="C158" t="s">
         <v>325</v>
@@ -18446,15 +18446,15 @@
         <v>19</v>
       </c>
       <c r="K158" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="159" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
+        <v>338</v>
+      </c>
+      <c r="B159" t="s">
         <v>339</v>
-      </c>
-      <c r="B159" t="s">
-        <v>340</v>
       </c>
       <c r="C159" t="s">
         <v>325</v>
@@ -18481,15 +18481,15 @@
         <v>19</v>
       </c>
       <c r="K159" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="160" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
+        <v>340</v>
+      </c>
+      <c r="B160" t="s">
         <v>341</v>
-      </c>
-      <c r="B160" t="s">
-        <v>342</v>
       </c>
       <c r="C160" t="s">
         <v>325</v>
@@ -18516,15 +18516,15 @@
         <v>19</v>
       </c>
       <c r="K160" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="161" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
+        <v>342</v>
+      </c>
+      <c r="B161" t="s">
         <v>343</v>
-      </c>
-      <c r="B161" t="s">
-        <v>344</v>
       </c>
       <c r="C161" t="s">
         <v>325</v>
@@ -18551,15 +18551,15 @@
         <v>19</v>
       </c>
       <c r="K161" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="162" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
+        <v>344</v>
+      </c>
+      <c r="B162" t="s">
         <v>345</v>
-      </c>
-      <c r="B162" t="s">
-        <v>346</v>
       </c>
       <c r="C162" t="s">
         <v>325</v>
@@ -18586,15 +18586,15 @@
         <v>19</v>
       </c>
       <c r="K162" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="163" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
+        <v>346</v>
+      </c>
+      <c r="B163" t="s">
         <v>347</v>
-      </c>
-      <c r="B163" t="s">
-        <v>348</v>
       </c>
       <c r="C163" t="s">
         <v>325</v>
@@ -18621,15 +18621,15 @@
         <v>19</v>
       </c>
       <c r="K163" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="164" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
+        <v>348</v>
+      </c>
+      <c r="B164" t="s">
         <v>349</v>
-      </c>
-      <c r="B164" t="s">
-        <v>350</v>
       </c>
       <c r="C164" t="s">
         <v>325</v>
@@ -18656,15 +18656,15 @@
         <v>19</v>
       </c>
       <c r="K164" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="165" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
+        <v>350</v>
+      </c>
+      <c r="B165" t="s">
         <v>351</v>
-      </c>
-      <c r="B165" t="s">
-        <v>352</v>
       </c>
       <c r="C165" t="s">
         <v>325</v>
@@ -18691,15 +18691,15 @@
         <v>19</v>
       </c>
       <c r="K165" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="166" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
+        <v>352</v>
+      </c>
+      <c r="B166" t="s">
         <v>353</v>
-      </c>
-      <c r="B166" t="s">
-        <v>354</v>
       </c>
       <c r="C166" t="s">
         <v>325</v>
@@ -18726,15 +18726,15 @@
         <v>19</v>
       </c>
       <c r="K166" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="167" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
+        <v>354</v>
+      </c>
+      <c r="B167" t="s">
         <v>355</v>
-      </c>
-      <c r="B167" t="s">
-        <v>356</v>
       </c>
       <c r="C167" t="s">
         <v>325</v>
@@ -18761,15 +18761,15 @@
         <v>19</v>
       </c>
       <c r="K167" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="168" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
+        <v>356</v>
+      </c>
+      <c r="B168" t="s">
         <v>357</v>
-      </c>
-      <c r="B168" t="s">
-        <v>358</v>
       </c>
       <c r="C168" t="s">
         <v>325</v>
@@ -18796,15 +18796,15 @@
         <v>19</v>
       </c>
       <c r="K168" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="169" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
+        <v>358</v>
+      </c>
+      <c r="B169" t="s">
         <v>359</v>
-      </c>
-      <c r="B169" t="s">
-        <v>360</v>
       </c>
       <c r="C169" t="s">
         <v>325</v>
@@ -18831,15 +18831,15 @@
         <v>19</v>
       </c>
       <c r="K169" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="170" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
+        <v>360</v>
+      </c>
+      <c r="B170" t="s">
         <v>361</v>
-      </c>
-      <c r="B170" t="s">
-        <v>362</v>
       </c>
       <c r="C170" t="s">
         <v>325</v>
@@ -18866,15 +18866,15 @@
         <v>19</v>
       </c>
       <c r="K170" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="171" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
+        <v>362</v>
+      </c>
+      <c r="B171" t="s">
         <v>363</v>
-      </c>
-      <c r="B171" t="s">
-        <v>364</v>
       </c>
       <c r="C171" t="s">
         <v>325</v>
@@ -18901,15 +18901,15 @@
         <v>19</v>
       </c>
       <c r="K171" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="172" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
+        <v>364</v>
+      </c>
+      <c r="B172" t="s">
         <v>365</v>
-      </c>
-      <c r="B172" t="s">
-        <v>366</v>
       </c>
       <c r="C172" t="s">
         <v>325</v>
@@ -18936,15 +18936,15 @@
         <v>19</v>
       </c>
       <c r="K172" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="173" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
+        <v>366</v>
+      </c>
+      <c r="B173" t="s">
         <v>367</v>
-      </c>
-      <c r="B173" t="s">
-        <v>368</v>
       </c>
       <c r="C173" t="s">
         <v>325</v>
@@ -18971,15 +18971,15 @@
         <v>19</v>
       </c>
       <c r="K173" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="174" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
+        <v>368</v>
+      </c>
+      <c r="B174" t="s">
         <v>369</v>
-      </c>
-      <c r="B174" t="s">
-        <v>370</v>
       </c>
       <c r="C174" t="s">
         <v>325</v>
@@ -19006,15 +19006,15 @@
         <v>19</v>
       </c>
       <c r="K174" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="175" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
+        <v>370</v>
+      </c>
+      <c r="B175" t="s">
         <v>371</v>
-      </c>
-      <c r="B175" t="s">
-        <v>372</v>
       </c>
       <c r="C175" t="s">
         <v>325</v>
@@ -19041,15 +19041,15 @@
         <v>19</v>
       </c>
       <c r="K175" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="176" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
+        <v>372</v>
+      </c>
+      <c r="B176" t="s">
         <v>373</v>
-      </c>
-      <c r="B176" t="s">
-        <v>374</v>
       </c>
       <c r="C176" t="s">
         <v>325</v>
@@ -19076,15 +19076,15 @@
         <v>19</v>
       </c>
       <c r="K176" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="177" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
+        <v>374</v>
+      </c>
+      <c r="B177" t="s">
         <v>375</v>
-      </c>
-      <c r="B177" t="s">
-        <v>376</v>
       </c>
       <c r="C177" t="s">
         <v>325</v>
@@ -19111,15 +19111,15 @@
         <v>19</v>
       </c>
       <c r="K177" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="178" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
+        <v>376</v>
+      </c>
+      <c r="B178" t="s">
         <v>377</v>
-      </c>
-      <c r="B178" t="s">
-        <v>378</v>
       </c>
       <c r="C178" t="s">
         <v>325</v>
@@ -19146,15 +19146,15 @@
         <v>19</v>
       </c>
       <c r="K178" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="179" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
+        <v>378</v>
+      </c>
+      <c r="B179" t="s">
         <v>379</v>
-      </c>
-      <c r="B179" t="s">
-        <v>380</v>
       </c>
       <c r="C179" t="s">
         <v>325</v>
@@ -19181,15 +19181,15 @@
         <v>19</v>
       </c>
       <c r="K179" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="180" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
+        <v>380</v>
+      </c>
+      <c r="B180" t="s">
         <v>381</v>
-      </c>
-      <c r="B180" t="s">
-        <v>382</v>
       </c>
       <c r="C180" t="s">
         <v>325</v>
@@ -19216,15 +19216,15 @@
         <v>19</v>
       </c>
       <c r="K180" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="181" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
+        <v>382</v>
+      </c>
+      <c r="B181" t="s">
         <v>383</v>
-      </c>
-      <c r="B181" t="s">
-        <v>384</v>
       </c>
       <c r="C181" t="s">
         <v>325</v>
@@ -19251,19 +19251,19 @@
         <v>19</v>
       </c>
       <c r="K181" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="182" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
+        <v>384</v>
+      </c>
+      <c r="B182" t="s">
         <v>385</v>
       </c>
-      <c r="B182" t="s">
+      <c r="C182" t="s">
         <v>386</v>
       </c>
-      <c r="C182" t="s">
-        <v>387</v>
-      </c>
       <c r="D182" t="s">
         <v>14</v>
       </c>
@@ -19286,18 +19286,18 @@
         <v>19</v>
       </c>
       <c r="K182" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="183" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
+        <v>387</v>
+      </c>
+      <c r="B183" t="s">
         <v>388</v>
       </c>
-      <c r="B183" t="s">
-        <v>389</v>
-      </c>
       <c r="C183" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D183" t="s">
         <v>14</v>
@@ -19321,18 +19321,18 @@
         <v>19</v>
       </c>
       <c r="K183" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="184" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
+        <v>389</v>
+      </c>
+      <c r="B184" t="s">
         <v>390</v>
       </c>
-      <c r="B184" t="s">
-        <v>391</v>
-      </c>
       <c r="C184" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D184" t="s">
         <v>14</v>
@@ -19356,18 +19356,18 @@
         <v>19</v>
       </c>
       <c r="K184" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="185" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
+        <v>391</v>
+      </c>
+      <c r="B185" t="s">
         <v>392</v>
       </c>
-      <c r="B185" t="s">
-        <v>393</v>
-      </c>
       <c r="C185" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D185" t="s">
         <v>14</v>
@@ -19391,18 +19391,18 @@
         <v>19</v>
       </c>
       <c r="K185" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="186" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
+        <v>393</v>
+      </c>
+      <c r="B186" t="s">
         <v>394</v>
       </c>
-      <c r="B186" t="s">
-        <v>395</v>
-      </c>
       <c r="C186" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D186" t="s">
         <v>14</v>
@@ -19426,18 +19426,18 @@
         <v>19</v>
       </c>
       <c r="K186" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="187" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
+        <v>395</v>
+      </c>
+      <c r="B187" t="s">
         <v>396</v>
       </c>
-      <c r="B187" t="s">
-        <v>397</v>
-      </c>
       <c r="C187" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D187" t="s">
         <v>14</v>
@@ -19461,18 +19461,18 @@
         <v>19</v>
       </c>
       <c r="K187" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="188" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
+        <v>397</v>
+      </c>
+      <c r="B188" t="s">
         <v>398</v>
       </c>
-      <c r="B188" t="s">
-        <v>399</v>
-      </c>
       <c r="C188" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D188" t="s">
         <v>14</v>
@@ -19496,42 +19496,42 @@
         <v>19</v>
       </c>
       <c r="K188" t="s">
-        <v>328</v>
+        <v>20</v>
       </c>
     </row>
     <row r="189" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
+        <v>399</v>
+      </c>
+      <c r="B189" t="s">
         <v>400</v>
       </c>
-      <c r="B189" t="s">
+      <c r="C189" t="s">
+        <v>386</v>
+      </c>
+      <c r="D189" t="s">
+        <v>14</v>
+      </c>
+      <c r="E189" t="s">
+        <v>15</v>
+      </c>
+      <c r="F189" t="s">
+        <v>16</v>
+      </c>
+      <c r="G189" t="s">
+        <v>17</v>
+      </c>
+      <c r="H189" t="s">
+        <v>18</v>
+      </c>
+      <c r="I189" t="s">
+        <v>19</v>
+      </c>
+      <c r="J189" t="s">
+        <v>19</v>
+      </c>
+      <c r="K189" t="s">
         <v>401</v>
-      </c>
-      <c r="C189" t="s">
-        <v>387</v>
-      </c>
-      <c r="D189" t="s">
-        <v>14</v>
-      </c>
-      <c r="E189" t="s">
-        <v>15</v>
-      </c>
-      <c r="F189" t="s">
-        <v>16</v>
-      </c>
-      <c r="G189" t="s">
-        <v>17</v>
-      </c>
-      <c r="H189" t="s">
-        <v>18</v>
-      </c>
-      <c r="I189" t="s">
-        <v>19</v>
-      </c>
-      <c r="J189" t="s">
-        <v>19</v>
-      </c>
-      <c r="K189" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="190" spans="1:11" x14ac:dyDescent="0.25">
@@ -19542,7 +19542,7 @@
         <v>403</v>
       </c>
       <c r="C190" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D190" t="s">
         <v>14</v>
@@ -19566,7 +19566,7 @@
         <v>19</v>
       </c>
       <c r="K190" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="191" spans="1:11" x14ac:dyDescent="0.25">
@@ -19577,7 +19577,7 @@
         <v>405</v>
       </c>
       <c r="C191" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D191" t="s">
         <v>14</v>
@@ -19601,7 +19601,7 @@
         <v>19</v>
       </c>
       <c r="K191" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="192" spans="1:11" x14ac:dyDescent="0.25">
@@ -19612,7 +19612,7 @@
         <v>407</v>
       </c>
       <c r="C192" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D192" t="s">
         <v>14</v>
@@ -19636,7 +19636,7 @@
         <v>19</v>
       </c>
       <c r="K192" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="193" spans="1:11" x14ac:dyDescent="0.25">
@@ -19647,7 +19647,7 @@
         <v>409</v>
       </c>
       <c r="C193" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D193" t="s">
         <v>14</v>
@@ -19671,7 +19671,7 @@
         <v>19</v>
       </c>
       <c r="K193" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="194" spans="1:11" x14ac:dyDescent="0.25">
@@ -19682,7 +19682,7 @@
         <v>411</v>
       </c>
       <c r="C194" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D194" t="s">
         <v>14</v>
@@ -19706,7 +19706,7 @@
         <v>19</v>
       </c>
       <c r="K194" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="195" spans="1:11" x14ac:dyDescent="0.25">
@@ -19717,7 +19717,7 @@
         <v>413</v>
       </c>
       <c r="C195" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D195" t="s">
         <v>14</v>
@@ -19741,7 +19741,7 @@
         <v>19</v>
       </c>
       <c r="K195" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="196" spans="1:11" x14ac:dyDescent="0.25">
@@ -19752,7 +19752,7 @@
         <v>415</v>
       </c>
       <c r="C196" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D196" t="s">
         <v>14</v>
@@ -19776,7 +19776,7 @@
         <v>19</v>
       </c>
       <c r="K196" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="197" spans="1:11" x14ac:dyDescent="0.25">
@@ -19787,7 +19787,7 @@
         <v>417</v>
       </c>
       <c r="C197" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D197" t="s">
         <v>14</v>
@@ -19811,7 +19811,7 @@
         <v>19</v>
       </c>
       <c r="K197" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="198" spans="1:11" x14ac:dyDescent="0.25">
@@ -19822,7 +19822,7 @@
         <v>419</v>
       </c>
       <c r="C198" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D198" t="s">
         <v>14</v>
@@ -19846,7 +19846,7 @@
         <v>19</v>
       </c>
       <c r="K198" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="199" spans="1:11" x14ac:dyDescent="0.25">
@@ -19857,7 +19857,7 @@
         <v>421</v>
       </c>
       <c r="C199" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D199" t="s">
         <v>14</v>
@@ -19881,7 +19881,7 @@
         <v>19</v>
       </c>
       <c r="K199" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="200" spans="1:11" x14ac:dyDescent="0.25">
@@ -19892,7 +19892,7 @@
         <v>423</v>
       </c>
       <c r="C200" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D200" t="s">
         <v>14</v>
@@ -19916,7 +19916,7 @@
         <v>19</v>
       </c>
       <c r="K200" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="201" spans="1:11" x14ac:dyDescent="0.25">
@@ -19927,7 +19927,7 @@
         <v>425</v>
       </c>
       <c r="C201" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D201" t="s">
         <v>14</v>
@@ -19951,7 +19951,7 @@
         <v>19</v>
       </c>
       <c r="K201" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="202" spans="1:11" x14ac:dyDescent="0.25">
@@ -19962,7 +19962,7 @@
         <v>427</v>
       </c>
       <c r="C202" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D202" t="s">
         <v>14</v>
@@ -19986,7 +19986,7 @@
         <v>19</v>
       </c>
       <c r="K202" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="203" spans="1:11" x14ac:dyDescent="0.25">
@@ -19997,7 +19997,7 @@
         <v>429</v>
       </c>
       <c r="C203" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D203" t="s">
         <v>14</v>
@@ -20021,7 +20021,7 @@
         <v>19</v>
       </c>
       <c r="K203" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="204" spans="1:11" x14ac:dyDescent="0.25">
@@ -20032,7 +20032,7 @@
         <v>431</v>
       </c>
       <c r="C204" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D204" t="s">
         <v>14</v>
@@ -20056,7 +20056,7 @@
         <v>19</v>
       </c>
       <c r="K204" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="205" spans="1:11" x14ac:dyDescent="0.25">
@@ -20067,7 +20067,7 @@
         <v>433</v>
       </c>
       <c r="C205" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D205" t="s">
         <v>14</v>
@@ -20091,7 +20091,7 @@
         <v>19</v>
       </c>
       <c r="K205" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="206" spans="1:11" x14ac:dyDescent="0.25">
@@ -20102,7 +20102,7 @@
         <v>435</v>
       </c>
       <c r="C206" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D206" t="s">
         <v>14</v>
@@ -20126,7 +20126,7 @@
         <v>19</v>
       </c>
       <c r="K206" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="207" spans="1:11" x14ac:dyDescent="0.25">
@@ -20137,7 +20137,7 @@
         <v>437</v>
       </c>
       <c r="C207" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D207" t="s">
         <v>14</v>
@@ -20161,7 +20161,7 @@
         <v>19</v>
       </c>
       <c r="K207" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="208" spans="1:11" x14ac:dyDescent="0.25">
@@ -20172,7 +20172,7 @@
         <v>439</v>
       </c>
       <c r="C208" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D208" t="s">
         <v>14</v>
@@ -20196,7 +20196,7 @@
         <v>19</v>
       </c>
       <c r="K208" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="209" spans="1:11" x14ac:dyDescent="0.25">
@@ -20207,7 +20207,7 @@
         <v>441</v>
       </c>
       <c r="C209" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D209" t="s">
         <v>14</v>
@@ -20231,7 +20231,7 @@
         <v>19</v>
       </c>
       <c r="K209" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="210" spans="1:11" x14ac:dyDescent="0.25">
@@ -20242,7 +20242,7 @@
         <v>443</v>
       </c>
       <c r="C210" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D210" t="s">
         <v>14</v>
@@ -20266,7 +20266,7 @@
         <v>19</v>
       </c>
       <c r="K210" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="211" spans="1:11" x14ac:dyDescent="0.25">
@@ -20277,7 +20277,7 @@
         <v>445</v>
       </c>
       <c r="C211" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D211" t="s">
         <v>14</v>
@@ -20301,7 +20301,7 @@
         <v>19</v>
       </c>
       <c r="K211" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="212" spans="1:11" x14ac:dyDescent="0.25">
@@ -20336,7 +20336,7 @@
         <v>19</v>
       </c>
       <c r="K212" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="213" spans="1:11" x14ac:dyDescent="0.25">
@@ -20371,7 +20371,7 @@
         <v>19</v>
       </c>
       <c r="K213" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="214" spans="1:11" x14ac:dyDescent="0.25">
@@ -20406,7 +20406,7 @@
         <v>19</v>
       </c>
       <c r="K214" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="215" spans="1:11" x14ac:dyDescent="0.25">
@@ -20441,7 +20441,7 @@
         <v>19</v>
       </c>
       <c r="K215" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="216" spans="1:11" x14ac:dyDescent="0.25">
@@ -20476,7 +20476,7 @@
         <v>19</v>
       </c>
       <c r="K216" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="217" spans="1:11" x14ac:dyDescent="0.25">
@@ -20511,7 +20511,7 @@
         <v>19</v>
       </c>
       <c r="K217" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="218" spans="1:11" x14ac:dyDescent="0.25">
@@ -20546,7 +20546,7 @@
         <v>19</v>
       </c>
       <c r="K218" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="219" spans="1:11" x14ac:dyDescent="0.25">
@@ -20581,7 +20581,7 @@
         <v>19</v>
       </c>
       <c r="K219" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="220" spans="1:11" x14ac:dyDescent="0.25">
@@ -20616,7 +20616,7 @@
         <v>19</v>
       </c>
       <c r="K220" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="221" spans="1:11" x14ac:dyDescent="0.25">
@@ -20651,7 +20651,7 @@
         <v>19</v>
       </c>
       <c r="K221" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="222" spans="1:11" x14ac:dyDescent="0.25">
@@ -20686,7 +20686,7 @@
         <v>19</v>
       </c>
       <c r="K222" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="223" spans="1:11" x14ac:dyDescent="0.25">
@@ -20721,7 +20721,7 @@
         <v>19</v>
       </c>
       <c r="K223" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="224" spans="1:11" x14ac:dyDescent="0.25">
@@ -20756,7 +20756,7 @@
         <v>19</v>
       </c>
       <c r="K224" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="225" spans="1:11" x14ac:dyDescent="0.25">
@@ -20791,7 +20791,7 @@
         <v>19</v>
       </c>
       <c r="K225" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="226" spans="1:11" x14ac:dyDescent="0.25">
@@ -20826,7 +20826,7 @@
         <v>19</v>
       </c>
       <c r="K226" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="227" spans="1:11" x14ac:dyDescent="0.25">
@@ -20861,7 +20861,7 @@
         <v>19</v>
       </c>
       <c r="K227" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="228" spans="1:11" x14ac:dyDescent="0.25">
@@ -20896,7 +20896,7 @@
         <v>19</v>
       </c>
       <c r="K228" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="229" spans="1:11" x14ac:dyDescent="0.25">
@@ -20931,7 +20931,7 @@
         <v>19</v>
       </c>
       <c r="K229" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="230" spans="1:11" x14ac:dyDescent="0.25">
@@ -20966,7 +20966,7 @@
         <v>19</v>
       </c>
       <c r="K230" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="231" spans="1:11" x14ac:dyDescent="0.25">
@@ -21001,7 +21001,7 @@
         <v>19</v>
       </c>
       <c r="K231" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="232" spans="1:11" x14ac:dyDescent="0.25">
@@ -21036,7 +21036,7 @@
         <v>19</v>
       </c>
       <c r="K232" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="233" spans="1:11" x14ac:dyDescent="0.25">
@@ -21071,7 +21071,7 @@
         <v>19</v>
       </c>
       <c r="K233" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="234" spans="1:11" x14ac:dyDescent="0.25">
@@ -21106,7 +21106,7 @@
         <v>19</v>
       </c>
       <c r="K234" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="235" spans="1:11" x14ac:dyDescent="0.25">
@@ -21141,7 +21141,7 @@
         <v>19</v>
       </c>
       <c r="K235" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="236" spans="1:11" x14ac:dyDescent="0.25">
@@ -21176,7 +21176,7 @@
         <v>19</v>
       </c>
       <c r="K236" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="237" spans="1:11" x14ac:dyDescent="0.25">
@@ -21211,7 +21211,7 @@
         <v>19</v>
       </c>
       <c r="K237" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="238" spans="1:11" x14ac:dyDescent="0.25">
@@ -21246,7 +21246,7 @@
         <v>19</v>
       </c>
       <c r="K238" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="239" spans="1:11" x14ac:dyDescent="0.25">
@@ -21281,7 +21281,7 @@
         <v>19</v>
       </c>
       <c r="K239" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="240" spans="1:11" x14ac:dyDescent="0.25">
@@ -21316,7 +21316,7 @@
         <v>19</v>
       </c>
       <c r="K240" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="241" spans="1:11" x14ac:dyDescent="0.25">
@@ -21351,7 +21351,7 @@
         <v>19</v>
       </c>
       <c r="K241" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="242" spans="1:11" x14ac:dyDescent="0.25">
@@ -21386,7 +21386,7 @@
         <v>19</v>
       </c>
       <c r="K242" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="243" spans="1:11" x14ac:dyDescent="0.25">
@@ -21421,7 +21421,7 @@
         <v>19</v>
       </c>
       <c r="K243" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="244" spans="1:11" x14ac:dyDescent="0.25">
@@ -21456,7 +21456,7 @@
         <v>19</v>
       </c>
       <c r="K244" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="245" spans="1:11" x14ac:dyDescent="0.25">
@@ -21491,7 +21491,7 @@
         <v>19</v>
       </c>
       <c r="K245" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="246" spans="1:11" x14ac:dyDescent="0.25">
@@ -21526,7 +21526,7 @@
         <v>19</v>
       </c>
       <c r="K246" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="247" spans="1:11" x14ac:dyDescent="0.25">
@@ -21561,7 +21561,7 @@
         <v>19</v>
       </c>
       <c r="K247" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="248" spans="1:11" x14ac:dyDescent="0.25">
@@ -21596,7 +21596,7 @@
         <v>19</v>
       </c>
       <c r="K248" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="249" spans="1:11" x14ac:dyDescent="0.25">
@@ -21631,7 +21631,7 @@
         <v>19</v>
       </c>
       <c r="K249" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="250" spans="1:11" x14ac:dyDescent="0.25">
@@ -21666,7 +21666,7 @@
         <v>19</v>
       </c>
       <c r="K250" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="251" spans="1:11" x14ac:dyDescent="0.25">
@@ -21701,7 +21701,7 @@
         <v>19</v>
       </c>
       <c r="K251" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="252" spans="1:11" x14ac:dyDescent="0.25">
@@ -21736,7 +21736,7 @@
         <v>19</v>
       </c>
       <c r="K252" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="253" spans="1:11" x14ac:dyDescent="0.25">
@@ -21771,7 +21771,7 @@
         <v>19</v>
       </c>
       <c r="K253" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="254" spans="1:11" x14ac:dyDescent="0.25">
@@ -21806,7 +21806,7 @@
         <v>19</v>
       </c>
       <c r="K254" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="255" spans="1:11" x14ac:dyDescent="0.25">
@@ -21841,7 +21841,7 @@
         <v>19</v>
       </c>
       <c r="K255" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="256" spans="1:11" x14ac:dyDescent="0.25">
@@ -21876,7 +21876,7 @@
         <v>19</v>
       </c>
       <c r="K256" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="257" spans="1:11" x14ac:dyDescent="0.25">
@@ -21911,7 +21911,7 @@
         <v>19</v>
       </c>
       <c r="K257" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="258" spans="1:11" x14ac:dyDescent="0.25">
@@ -21946,7 +21946,7 @@
         <v>19</v>
       </c>
       <c r="K258" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="259" spans="1:11" x14ac:dyDescent="0.25">
@@ -21981,7 +21981,7 @@
         <v>19</v>
       </c>
       <c r="K259" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="260" spans="1:11" x14ac:dyDescent="0.25">
@@ -22016,7 +22016,7 @@
         <v>19</v>
       </c>
       <c r="K260" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="261" spans="1:11" x14ac:dyDescent="0.25">
@@ -22051,7 +22051,7 @@
         <v>19</v>
       </c>
       <c r="K261" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="262" spans="1:11" x14ac:dyDescent="0.25">
@@ -22086,7 +22086,7 @@
         <v>19</v>
       </c>
       <c r="K262" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="263" spans="1:11" x14ac:dyDescent="0.25">
@@ -22121,7 +22121,7 @@
         <v>19</v>
       </c>
       <c r="K263" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="264" spans="1:11" x14ac:dyDescent="0.25">
@@ -22156,7 +22156,7 @@
         <v>19</v>
       </c>
       <c r="K264" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="265" spans="1:11" x14ac:dyDescent="0.25">
@@ -22191,7 +22191,7 @@
         <v>19</v>
       </c>
       <c r="K265" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="266" spans="1:11" x14ac:dyDescent="0.25">
@@ -22226,7 +22226,7 @@
         <v>19</v>
       </c>
       <c r="K266" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="267" spans="1:11" x14ac:dyDescent="0.25">
@@ -22261,7 +22261,7 @@
         <v>19</v>
       </c>
       <c r="K267" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="268" spans="1:11" x14ac:dyDescent="0.25">
@@ -22296,7 +22296,7 @@
         <v>19</v>
       </c>
       <c r="K268" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="269" spans="1:11" x14ac:dyDescent="0.25">
@@ -22331,7 +22331,7 @@
         <v>19</v>
       </c>
       <c r="K269" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="270" spans="1:11" x14ac:dyDescent="0.25">
@@ -22366,7 +22366,7 @@
         <v>19</v>
       </c>
       <c r="K270" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="271" spans="1:11" x14ac:dyDescent="0.25">
@@ -22401,7 +22401,7 @@
         <v>19</v>
       </c>
       <c r="K271" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="272" spans="1:11" x14ac:dyDescent="0.25">
@@ -22436,7 +22436,7 @@
         <v>19</v>
       </c>
       <c r="K272" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="273" spans="1:11" x14ac:dyDescent="0.25">
@@ -22471,7 +22471,7 @@
         <v>19</v>
       </c>
       <c r="K273" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="274" spans="1:11" x14ac:dyDescent="0.25">
@@ -22506,7 +22506,7 @@
         <v>19</v>
       </c>
       <c r="K274" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="275" spans="1:11" x14ac:dyDescent="0.25">
@@ -22541,7 +22541,7 @@
         <v>19</v>
       </c>
       <c r="K275" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="276" spans="1:11" x14ac:dyDescent="0.25">
@@ -22576,7 +22576,7 @@
         <v>19</v>
       </c>
       <c r="K276" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="277" spans="1:11" x14ac:dyDescent="0.25">
@@ -22611,7 +22611,7 @@
         <v>19</v>
       </c>
       <c r="K277" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="278" spans="1:11" x14ac:dyDescent="0.25">
@@ -22646,7 +22646,7 @@
         <v>19</v>
       </c>
       <c r="K278" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="279" spans="1:11" x14ac:dyDescent="0.25">
@@ -22681,7 +22681,7 @@
         <v>19</v>
       </c>
       <c r="K279" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="280" spans="1:11" x14ac:dyDescent="0.25">
@@ -22716,7 +22716,7 @@
         <v>19</v>
       </c>
       <c r="K280" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="281" spans="1:11" x14ac:dyDescent="0.25">
@@ -22751,7 +22751,7 @@
         <v>19</v>
       </c>
       <c r="K281" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="282" spans="1:11" x14ac:dyDescent="0.25">
@@ -22786,7 +22786,7 @@
         <v>19</v>
       </c>
       <c r="K282" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="283" spans="1:11" x14ac:dyDescent="0.25">
@@ -22821,7 +22821,7 @@
         <v>19</v>
       </c>
       <c r="K283" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="284" spans="1:11" x14ac:dyDescent="0.25">
@@ -22856,7 +22856,7 @@
         <v>19</v>
       </c>
       <c r="K284" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="285" spans="1:11" x14ac:dyDescent="0.25">
@@ -22891,7 +22891,7 @@
         <v>19</v>
       </c>
       <c r="K285" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="286" spans="1:11" x14ac:dyDescent="0.25">
@@ -22926,7 +22926,7 @@
         <v>19</v>
       </c>
       <c r="K286" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="287" spans="1:11" x14ac:dyDescent="0.25">
@@ -22961,7 +22961,7 @@
         <v>19</v>
       </c>
       <c r="K287" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="288" spans="1:11" x14ac:dyDescent="0.25">
@@ -22996,7 +22996,7 @@
         <v>19</v>
       </c>
       <c r="K288" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="289" spans="1:11" x14ac:dyDescent="0.25">
@@ -23031,7 +23031,7 @@
         <v>19</v>
       </c>
       <c r="K289" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="290" spans="1:11" x14ac:dyDescent="0.25">
@@ -23066,7 +23066,7 @@
         <v>19</v>
       </c>
       <c r="K290" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="291" spans="1:11" x14ac:dyDescent="0.25">
@@ -23101,7 +23101,7 @@
         <v>19</v>
       </c>
       <c r="K291" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="292" spans="1:11" x14ac:dyDescent="0.25">
@@ -23136,7 +23136,7 @@
         <v>19</v>
       </c>
       <c r="K292" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="293" spans="1:11" x14ac:dyDescent="0.25">
@@ -23171,7 +23171,7 @@
         <v>19</v>
       </c>
       <c r="K293" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="294" spans="1:11" x14ac:dyDescent="0.25">
@@ -23206,7 +23206,7 @@
         <v>19</v>
       </c>
       <c r="K294" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="295" spans="1:11" x14ac:dyDescent="0.25">
@@ -23241,7 +23241,7 @@
         <v>19</v>
       </c>
       <c r="K295" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="296" spans="1:11" x14ac:dyDescent="0.25">
@@ -23276,7 +23276,7 @@
         <v>19</v>
       </c>
       <c r="K296" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="297" spans="1:11" x14ac:dyDescent="0.25">
@@ -23311,7 +23311,7 @@
         <v>19</v>
       </c>
       <c r="K297" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="298" spans="1:11" x14ac:dyDescent="0.25">
@@ -23346,7 +23346,7 @@
         <v>19</v>
       </c>
       <c r="K298" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="299" spans="1:11" x14ac:dyDescent="0.25">
@@ -23381,7 +23381,7 @@
         <v>19</v>
       </c>
       <c r="K299" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="300" spans="1:11" x14ac:dyDescent="0.25">
@@ -23416,7 +23416,7 @@
         <v>19</v>
       </c>
       <c r="K300" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
     <row r="301" spans="1:11" x14ac:dyDescent="0.25">
@@ -23451,7 +23451,7 @@
         <v>19</v>
       </c>
       <c r="K301" t="s">
-        <v>328</v>
+        <v>401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>